<commit_message>
Fill IPO sizes for Acutaas Chemicals (ex-Ami Organics) and Archit Nuwood
</commit_message>
<xml_diff>
--- a/Issue_Size_List_with_IPO_Size_notes.xlsx
+++ b/Issue_Size_List_with_IPO_Size_notes.xlsx
@@ -8951,30 +8951,64 @@
           <t>Equity</t>
         </is>
       </c>
-      <c r="F115" s="5" t="n"/>
-      <c r="G115" s="7" t="n"/>
-      <c r="H115" s="7" t="n"/>
-      <c r="I115" s="7" t="n"/>
-      <c r="J115" s="5" t="n"/>
-      <c r="K115" s="7" t="n"/>
-      <c r="L115" s="6" t="n"/>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>MainBoard</t>
+        </is>
+      </c>
+      <c r="G115" s="7" t="n">
+        <v>569.64</v>
+      </c>
+      <c r="H115" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="I115" s="7" t="n">
+        <v>369.64</v>
+      </c>
+      <c r="J115" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K115" s="7" t="n">
+        <v>610</v>
+      </c>
+      <c r="L115" s="6" t="n">
+        <v>44453</v>
+      </c>
       <c r="M115" s="7" t="n"/>
       <c r="N115" s="7" t="n"/>
-      <c r="O115" s="5" t="n"/>
-      <c r="P115" s="5" t="n"/>
+      <c r="O115" s="5" t="inlineStr">
+        <is>
+          <t>Chemicals</t>
+        </is>
+      </c>
+      <c r="P115" s="5" t="inlineStr">
+        <is>
+          <t>INE00FF01025</t>
+        </is>
+      </c>
       <c r="Q115" s="5" t="n"/>
-      <c r="R115" s="5" t="n"/>
+      <c r="R115" s="5" t="inlineStr">
+        <is>
+          <t>543349</t>
+        </is>
+      </c>
       <c r="S115" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Web search (former name)</t>
         </is>
       </c>
       <c r="T115" s="5" t="inlineStr">
         <is>
-          <t>IPO exists (missed by source) — Acutaas Chemicals is the former Ami Organics, which held a Rs 569.64 Cr IPO (Rs 200 Cr fresh issue plus Rs 369.64 Cr offer for sale, priced at Rs 610) and listed on 14 Sep 2021; the source missed it because of the name change. Source: https://www.chittorgarh.com/ipo/ami-organics-ipo/1143/</t>
-        </is>
-      </c>
-      <c r="U115" s="5" t="n"/>
+          <t>IPO filled manually: listed as Ami Organics Ltd (renamed Acutaas Chemicals); book-built IPO of Rs 569.64 Cr (Rs 200 Cr fresh + Rs 369.64 Cr OFS) at Rs 610, 1-3 Sep 2021, subscribed 64.54x, listed NSE/BSE 14 Sep 2021. Source missed it due to the name change.</t>
+        </is>
+      </c>
+      <c r="U115" s="5" t="inlineStr">
+        <is>
+          <t>https://www.chittorgarh.com/ipo/ami-organics-ipo/1143/</t>
+        </is>
+      </c>
     </row>
     <row r="116" hidden="1">
       <c r="A116" s="2" t="inlineStr">
@@ -32838,30 +32872,60 @@
           <t>Equity</t>
         </is>
       </c>
-      <c r="F444" s="5" t="n"/>
-      <c r="G444" s="7" t="n"/>
-      <c r="H444" s="7" t="n"/>
-      <c r="I444" s="7" t="n"/>
-      <c r="J444" s="5" t="n"/>
-      <c r="K444" s="7" t="n"/>
-      <c r="L444" s="6" t="n"/>
+      <c r="F444" s="5" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="G444" s="7" t="n">
+        <v>168.48</v>
+      </c>
+      <c r="H444" s="7" t="n">
+        <v>168.48</v>
+      </c>
+      <c r="I444" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J444" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K444" s="7" t="n">
+        <v>270</v>
+      </c>
+      <c r="L444" s="6" t="n">
+        <v>45541</v>
+      </c>
       <c r="M444" s="7" t="n"/>
       <c r="N444" s="7" t="n"/>
-      <c r="O444" s="5" t="n"/>
-      <c r="P444" s="5" t="n"/>
+      <c r="O444" s="5" t="inlineStr">
+        <is>
+          <t>Wood Panels (MDF/HDF)</t>
+        </is>
+      </c>
+      <c r="P444" s="5" t="inlineStr">
+        <is>
+          <t>INE0RH401013</t>
+        </is>
+      </c>
       <c r="Q444" s="5" t="n"/>
       <c r="R444" s="5" t="n"/>
       <c r="S444" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>Web search</t>
         </is>
       </c>
       <c r="T444" s="5" t="inlineStr">
         <is>
-          <t>IPO exists (missed by source) — Archit Nuwood Industries did hold an IPO, a book-built issue of 62.40 lakh shares at Rs 257-270 (about Rs 168.48 Cr at the upper band), open 30 Aug to 3 Sep 2024, and listed on BSE SME on 6 Sep 2024. [confidence: medium] Source: https://www.chittorgarh.com/ipo_faqs/archit-nuwood-industries-ipo/1823/</t>
-        </is>
-      </c>
-      <c r="U444" s="5" t="n"/>
+          <t>IPO filled manually: BSE SME book-built issue of 62.40 lakh shares (fresh issue only) at Rs 257-270, 30 Aug-3 Sep 2024, listed BSE SME 6 Sep 2024; size taken at upper band Rs 270. Caveat: a pre-open report said the issue was delayed by exchange queries and no subscription figures were found, so verify the final issue price/size.</t>
+        </is>
+      </c>
+      <c r="U444" s="5" t="inlineStr">
+        <is>
+          <t>https://www.chittorgarh.com/ipo_news/archit-nuwood-industries-ipo/1823/</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">

</xml_diff>